<commit_message>
update dataset and config files
</commit_message>
<xml_diff>
--- a/data/raw/vocab_database.xlsx
+++ b/data/raw/vocab_database.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -450,7 +450,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -465,7 +465,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -480,7 +480,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -495,7 +495,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -525,7 +525,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -540,7 +540,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -555,7 +555,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -600,7 +600,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -615,7 +615,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -660,7 +660,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -690,7 +690,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -705,7 +705,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -720,7 +720,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -735,7 +735,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -780,7 +780,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -810,7 +810,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -840,7 +840,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -885,7 +885,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -900,7 +900,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -915,7 +915,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -960,7 +960,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -990,7 +990,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1005,7 +1005,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1020,7 +1020,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1095,7 +1095,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1110,7 +1110,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1125,7 +1125,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1140,7 +1140,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1185,7 +1185,7 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1200,7 +1200,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -1230,7 +1230,7 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1245,7 +1245,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -1260,7 +1260,7 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -1320,7 +1320,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>

</xml_diff>